<commit_message>
fix: update deprecated Gemini API model to gemini-3.8-flash in chat service and agent to restore AI responses
</commit_message>
<xml_diff>
--- a/SentinelMCP_Dataset_Clean.xlsx
+++ b/SentinelMCP_Dataset_Clean.xlsx
@@ -7069,16 +7069,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>96.06</v>
+        <v>78.73999999999999</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>93.83</v>
+        <v>66.67</v>
       </c>
       <c r="E4" t="n">
-        <v>96.81999999999999</v>
+        <v>80</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>

</xml_diff>